<commit_message>
atualiza volumes loa com ppo - 11092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
+++ b/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
@@ -62897,7 +62897,7 @@
         </is>
       </c>
       <c r="U905" t="n">
-        <v>565584854</v>
+        <v>579244576</v>
       </c>
       <c r="V905" t="n">
         <v>2027</v>
@@ -63449,7 +63449,7 @@
         </is>
       </c>
       <c r="U913" t="n">
-        <v>215645933</v>
+        <v>220854106</v>
       </c>
       <c r="V913" t="n">
         <v>2027</v>
@@ -63932,7 +63932,7 @@
         </is>
       </c>
       <c r="U920" t="n">
-        <v>99282753</v>
+        <v>101680580</v>
       </c>
       <c r="V920" t="n">
         <v>2027</v>
@@ -65795,7 +65795,7 @@
         </is>
       </c>
       <c r="U947" t="n">
-        <v>1131169707</v>
+        <v>1186551659</v>
       </c>
       <c r="V947" t="n">
         <v>2027</v>

</xml_diff>